<commit_message>
🤖 Actualización automática diaria [GitHub Actions]
</commit_message>
<xml_diff>
--- a/Precios_Metales_COP.xlsx
+++ b/Precios_Metales_COP.xlsx
@@ -22774,13 +22774,13 @@
         <v>46275</v>
       </c>
       <c r="B489" s="19" t="n">
-        <v>4416</v>
+        <v>4364.5</v>
       </c>
       <c r="C489" s="19" t="n">
-        <v>67.94200134277344</v>
+        <v>64.28399658203125</v>
       </c>
       <c r="D489" s="19" t="n">
-        <v>3087.64990234375</v>
+        <v>3101.550048828125</v>
       </c>
       <c r="E489" s="20">
         <f>ROUND((B489/31.1034768)*D489, 2)</f>
@@ -22804,13 +22804,13 @@
         <v>46276</v>
       </c>
       <c r="B490" s="15" t="n">
-        <v>4364.2001953125</v>
+        <v>4390</v>
       </c>
       <c r="C490" s="15" t="n">
-        <v>64.125</v>
+        <v>65.01999664306641</v>
       </c>
       <c r="D490" s="15" t="n">
-        <v>3087.64990234375</v>
+        <v>3082.739990234375</v>
       </c>
       <c r="E490" s="16">
         <f>ROUND((B490/31.1034768)*D490, 2)</f>

</xml_diff>